<commit_message>
Atualiza planilha com propostas e descontos
</commit_message>
<xml_diff>
--- a/dados/leiloes_rodovias.xlsx
+++ b/dados/leiloes_rodovias.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notas" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'leiloes'!$A$1:$V$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'leiloes'!$A$1:$AC$23</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="0.00000"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
-    <numFmt numFmtId="166" formatCode="#,##0.0"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,15 +63,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -436,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V23"/>
+  <dimension ref="A1:AC23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -461,6 +466,7 @@
     <col width="12" customWidth="1" min="20" max="20"/>
     <col width="50" customWidth="1" min="21" max="21"/>
     <col width="60" customWidth="1" min="22" max="22"/>
+    <col width="50" customWidth="1" min="27" max="27"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -566,10 +572,45 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
+          <t>vdma_contagem</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>pct_caminhoes</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>pct_pesados</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>vdma_equiv_pracas_ano1</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>cresc_trafego_aa</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>fuga_pct</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>estudo_demanda</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
           <t>observacao</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="AC1" s="1" t="inlineStr">
         <is>
           <t>fonte</t>
         </is>
@@ -604,7 +645,7 @@
       <c r="F2" t="n">
         <v>30</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="G2" s="6" t="n">
         <v>473.01</v>
       </c>
       <c r="H2" s="3" t="n">
@@ -616,10 +657,10 @@
       <c r="J2" s="4" t="n">
         <v>0.0847</v>
       </c>
-      <c r="K2" s="5" t="n">
+      <c r="K2" s="7" t="n">
         <v>0.0872</v>
       </c>
-      <c r="L2" s="5" t="n">
+      <c r="L2" s="7" t="n">
         <v>0.1221</v>
       </c>
       <c r="M2" t="inlineStr">
@@ -640,12 +681,18 @@
       <c r="S2" s="4" t="n">
         <v>0.1825</v>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="U2" s="8" t="n"/>
+      <c r="V2" s="9" t="n"/>
+      <c r="W2" s="9" t="n"/>
+      <c r="X2" s="8" t="n"/>
+      <c r="Y2" s="9" t="n"/>
+      <c r="Z2" s="9" t="n"/>
+      <c r="AB2" t="inlineStr">
         <is>
           <t>EPR ofereceu 8,30%; nº total de propostas a verificar</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="AC2" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-277-373-376-476-pr-e-pr-418-423-427 ; https://www.poder360.com.br/governo/grupo-patria-vence-leilao-rodoviario-do-lote-1-parana/</t>
         </is>
@@ -680,7 +727,7 @@
       <c r="F3" t="n">
         <v>30</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="G3" s="6" t="n">
         <v>604.66</v>
       </c>
       <c r="H3" s="3" t="n">
@@ -692,10 +739,10 @@
       <c r="J3" s="4" t="n">
         <v>0.0847</v>
       </c>
-      <c r="K3" s="5" t="n">
+      <c r="K3" s="7" t="n">
         <v>0.1191</v>
       </c>
-      <c r="L3" s="5" t="n">
+      <c r="L3" s="7" t="n">
         <v>0.1667</v>
       </c>
       <c r="M3" t="inlineStr">
@@ -719,12 +766,18 @@
       <c r="T3" t="n">
         <v>1</v>
       </c>
-      <c r="U3" t="inlineStr">
+      <c r="U3" s="8" t="n"/>
+      <c r="V3" s="9" t="n"/>
+      <c r="W3" s="9" t="n"/>
+      <c r="X3" s="8" t="n"/>
+      <c r="Y3" s="9" t="n"/>
+      <c r="Z3" s="9" t="n"/>
+      <c r="AB3" t="inlineStr">
         <is>
           <t>proposta única</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="AC3" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/2br-153-277-369-pr-e-pr-092-151-239-407-408-411-508-804-855 ; https://exame.com/brasil/lote-2-de-rodovias-do-parana-e-arrematado-em-leilao-com-so-1-interessado</t>
         </is>
@@ -759,7 +812,7 @@
       <c r="F4" t="n">
         <v>30</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="G4" s="6" t="n">
         <v>303.4</v>
       </c>
       <c r="H4" s="3" t="n">
@@ -771,10 +824,10 @@
       <c r="J4" s="4" t="n">
         <v>0.1197</v>
       </c>
-      <c r="K4" s="5" t="n">
+      <c r="K4" s="7" t="n">
         <v>0.1821</v>
       </c>
-      <c r="L4" s="5" t="n">
+      <c r="L4" s="7" t="n">
         <v>0.2549</v>
       </c>
       <c r="M4" t="inlineStr">
@@ -807,12 +860,18 @@
       <c r="T4" t="n">
         <v>2</v>
       </c>
-      <c r="U4" t="inlineStr">
+      <c r="U4" s="8" t="n"/>
+      <c r="V4" s="9" t="n"/>
+      <c r="W4" s="9" t="n"/>
+      <c r="X4" s="8" t="n"/>
+      <c r="Y4" s="9" t="n"/>
+      <c r="Z4" s="9" t="n"/>
+      <c r="AB4" t="inlineStr">
         <is>
           <t>1ª tentativa (nov/2023) sem propostas</t>
         </is>
       </c>
-      <c r="V4" t="inlineStr">
+      <c r="AC4" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-381-mg</t>
         </is>
@@ -847,7 +906,7 @@
       <c r="F5" t="n">
         <v>30</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="G5" s="6" t="n">
         <v>594.8</v>
       </c>
       <c r="H5" s="3" t="n">
@@ -859,10 +918,10 @@
       <c r="J5" s="4" t="n">
         <v>0.0921</v>
       </c>
-      <c r="K5" s="5" t="n">
+      <c r="K5" s="7" t="n">
         <v>0.124</v>
       </c>
-      <c r="L5" s="5" t="n">
+      <c r="L5" s="7" t="n">
         <v>0.1612</v>
       </c>
       <c r="M5" t="inlineStr">
@@ -884,12 +943,18 @@
       <c r="T5" t="n">
         <v>4</v>
       </c>
-      <c r="U5" t="inlineStr">
+      <c r="U5" s="8" t="n"/>
+      <c r="V5" s="9" t="n"/>
+      <c r="W5" s="9" t="n"/>
+      <c r="X5" s="8" t="n"/>
+      <c r="Y5" s="9" t="n"/>
+      <c r="Z5" s="9" t="n"/>
+      <c r="AB5" t="inlineStr">
         <is>
           <t>desconto a verificar (critério inclui outorga)</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr">
+      <c r="AC5" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-040-go-mg-rota-dos-cristais</t>
         </is>
@@ -924,7 +989,7 @@
       <c r="F6" t="n">
         <v>30</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="G6" s="6" t="n">
         <v>438.9</v>
       </c>
       <c r="H6" s="3" t="n">
@@ -936,10 +1001,10 @@
       <c r="J6" s="4" t="n">
         <v>0.0921</v>
       </c>
-      <c r="K6" s="5" t="n">
+      <c r="K6" s="7" t="n">
         <v>0.13969</v>
       </c>
-      <c r="L6" s="5" t="n">
+      <c r="L6" s="7" t="n">
         <v>0.1816</v>
       </c>
       <c r="M6" t="inlineStr">
@@ -960,8 +1025,13 @@
       <c r="S6" s="4" t="n">
         <v>0.153</v>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr">
+      <c r="U6" s="8" t="n"/>
+      <c r="V6" s="9" t="n"/>
+      <c r="W6" s="9" t="n"/>
+      <c r="X6" s="8" t="n"/>
+      <c r="Y6" s="9" t="n"/>
+      <c r="Z6" s="9" t="n"/>
+      <c r="AC6" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovia-br-262-mg-rota-do-zebu</t>
         </is>
@@ -996,7 +1066,7 @@
       <c r="F7" t="n">
         <v>30</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="G7" s="6" t="n">
         <v>569.75</v>
       </c>
       <c r="H7" s="3" t="n">
@@ -1008,10 +1078,10 @@
       <c r="J7" s="4" t="n">
         <v>0.1064</v>
       </c>
-      <c r="K7" s="5" t="n">
+      <c r="K7" s="7" t="n">
         <v>0.1459</v>
       </c>
-      <c r="L7" s="5" t="n">
+      <c r="L7" s="7" t="n">
         <v>0.20435</v>
       </c>
       <c r="M7" t="inlineStr">
@@ -1041,8 +1111,13 @@
       <c r="T7" t="n">
         <v>4</v>
       </c>
-      <c r="U7" t="inlineStr"/>
-      <c r="V7" t="inlineStr">
+      <c r="U7" s="8" t="n"/>
+      <c r="V7" s="9" t="n"/>
+      <c r="W7" s="9" t="n"/>
+      <c r="X7" s="8" t="n"/>
+      <c r="Y7" s="9" t="n"/>
+      <c r="Z7" s="9" t="n"/>
+      <c r="AC7" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-369-373-376-pr-e-pr-090-170-323-445</t>
         </is>
@@ -1077,7 +1152,7 @@
       <c r="F8" t="n">
         <v>30</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="G8" s="6" t="n">
         <v>426.2</v>
       </c>
       <c r="H8" s="3" t="n">
@@ -1089,10 +1164,10 @@
       <c r="J8" s="4" t="n">
         <v>0.09080000000000001</v>
       </c>
-      <c r="K8" s="5" t="n">
+      <c r="K8" s="7" t="n">
         <v>0.1017</v>
       </c>
-      <c r="L8" s="5" t="n">
+      <c r="L8" s="7" t="n">
         <v>0.1322</v>
       </c>
       <c r="M8" t="inlineStr">
@@ -1116,12 +1191,18 @@
       <c r="T8" t="n">
         <v>4</v>
       </c>
-      <c r="U8" t="inlineStr">
+      <c r="U8" s="8" t="n"/>
+      <c r="V8" s="9" t="n"/>
+      <c r="W8" s="9" t="n"/>
+      <c r="X8" s="8" t="n"/>
+      <c r="Y8" s="9" t="n"/>
+      <c r="Z8" s="9" t="n"/>
+      <c r="AB8" t="inlineStr">
         <is>
           <t>página da ANTT diz 12/12/2025, mas a homologação é de 17/01/2025: provável 2024; texto cita 452,7 km</t>
         </is>
       </c>
-      <c r="V8" t="inlineStr">
+      <c r="AC8" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/bndes-cn1-centro-oeste-norte</t>
         </is>
@@ -1156,7 +1237,7 @@
       <c r="F9" t="n">
         <v>30</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="G9" s="6" t="n">
         <v>662.1</v>
       </c>
       <c r="H9" s="3" t="n">
@@ -1168,10 +1249,10 @@
       <c r="J9" s="4" t="n">
         <v>0.1064</v>
       </c>
-      <c r="K9" s="5" t="n">
+      <c r="K9" s="7" t="n">
         <v>0.1758</v>
       </c>
-      <c r="L9" s="5" t="n">
+      <c r="L9" s="7" t="n">
         <v>0.2461</v>
       </c>
       <c r="M9" t="inlineStr">
@@ -1201,8 +1282,13 @@
       <c r="T9" t="n">
         <v>4</v>
       </c>
-      <c r="U9" t="inlineStr"/>
-      <c r="V9" t="inlineStr">
+      <c r="U9" s="8" t="n"/>
+      <c r="V9" s="9" t="n"/>
+      <c r="W9" s="9" t="n"/>
+      <c r="X9" s="8" t="n"/>
+      <c r="Y9" s="9" t="n"/>
+      <c r="Z9" s="9" t="n"/>
+      <c r="AC9" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovias-integradas-do-parana-lote-6</t>
         </is>
@@ -1237,7 +1323,7 @@
       <c r="F10" t="n">
         <v>30</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="G10" s="6" t="n">
         <v>686.7</v>
       </c>
       <c r="H10" s="3" t="n">
@@ -1249,10 +1335,10 @@
       <c r="J10" s="4" t="n">
         <v>0.1117</v>
       </c>
-      <c r="K10" s="5" t="n">
+      <c r="K10" s="7" t="n">
         <v>0.1911</v>
       </c>
-      <c r="L10" s="5" t="n">
+      <c r="L10" s="7" t="n">
         <v>0.2485</v>
       </c>
       <c r="M10" t="inlineStr">
@@ -1285,12 +1371,18 @@
       <c r="T10" t="n">
         <v>1</v>
       </c>
-      <c r="U10" t="inlineStr">
+      <c r="U10" s="8" t="n"/>
+      <c r="V10" s="9" t="n"/>
+      <c r="W10" s="9" t="n"/>
+      <c r="X10" s="8" t="n"/>
+      <c r="Y10" s="9" t="n"/>
+      <c r="Z10" s="9" t="n"/>
+      <c r="AB10" t="inlineStr">
         <is>
           <t>NeoFeed: 'apenas um concorrente'</t>
         </is>
       </c>
-      <c r="V10" t="inlineStr">
+      <c r="AC10" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/bndes-cn5-centro-oeste-norte ; https://neofeed.com.br/negocios/apenas-um-concorrente-e-pedagio-caro-a-decepcao-no-primeiro-de-15-leiloes-rodoviarios-do-ano/</t>
         </is>
@@ -1325,7 +1417,7 @@
       <c r="F11" t="n">
         <v>30</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="G11" s="6" t="n">
         <v>218.9</v>
       </c>
       <c r="H11" s="3" t="n">
@@ -1337,10 +1429,10 @@
       <c r="J11" s="4" t="n">
         <v>0.1117</v>
       </c>
-      <c r="K11" s="5" t="n">
+      <c r="K11" s="7" t="n">
         <v>0.3551</v>
       </c>
-      <c r="L11" s="5" t="n"/>
+      <c r="L11" s="7" t="n"/>
       <c r="M11" t="inlineStr">
         <is>
           <t>jan/23</t>
@@ -1368,12 +1460,18 @@
       <c r="T11" t="n">
         <v>3</v>
       </c>
-      <c r="U11" t="inlineStr">
+      <c r="U11" s="8" t="n"/>
+      <c r="V11" s="9" t="n"/>
+      <c r="W11" s="9" t="n"/>
+      <c r="X11" s="8" t="n"/>
+      <c r="Y11" s="9" t="n"/>
+      <c r="Z11" s="9" t="n"/>
+      <c r="AB11" t="inlineStr">
         <is>
           <t>tarifa única por km</t>
         </is>
       </c>
-      <c r="V11" t="inlineStr">
+      <c r="AC11" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/BR-040-495-MG-RJ-JF-RIO</t>
         </is>
@@ -1405,12 +1503,12 @@
           <t>08/05/2025</t>
         </is>
       </c>
-      <c r="G12" s="2" t="n"/>
+      <c r="G12" s="6" t="n"/>
       <c r="H12" s="3" t="n"/>
       <c r="I12" s="3" t="n"/>
       <c r="J12" s="4" t="n"/>
-      <c r="K12" s="5" t="n"/>
-      <c r="L12" s="5" t="n"/>
+      <c r="K12" s="7" t="n"/>
+      <c r="L12" s="7" t="n"/>
       <c r="M12" t="inlineStr">
         <is>
           <t>n/d</t>
@@ -1430,12 +1528,18 @@
       <c r="T12" t="n">
         <v>4</v>
       </c>
-      <c r="U12" t="inlineStr">
+      <c r="U12" s="8" t="n"/>
+      <c r="V12" s="9" t="n"/>
+      <c r="W12" s="9" t="n"/>
+      <c r="X12" s="8" t="n"/>
+      <c r="Y12" s="9" t="n"/>
+      <c r="Z12" s="9" t="n"/>
+      <c r="AB12" t="inlineStr">
         <is>
           <t>projeto do governo do MS; 1º colocado (K-Infra/Galápagos, 9%) desclassificado; dados a buscar</t>
         </is>
       </c>
-      <c r="V12" t="inlineStr">
+      <c r="AC12" t="inlineStr">
         <is>
           <t>https://www.demarest.com.br/consorcio-da-xp-assume-rota-da-celulose-apos-desclassificacao-de-rival/ ; https://istoedinheiro.com.br/kinfra-e-galapagos-arrematam-rota-da-celulose-com-desconto-de-9-sobre-tarifa-basica</t>
         </is>
@@ -1470,7 +1574,7 @@
       <c r="F13" t="n">
         <v>30</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="G13" s="6" t="n">
         <v>490.06</v>
       </c>
       <c r="H13" s="3" t="n">
@@ -1482,10 +1586,10 @@
       <c r="J13" s="4" t="n">
         <v>0.0999</v>
       </c>
-      <c r="K13" s="5" t="n">
+      <c r="K13" s="7" t="n">
         <v>0.1627</v>
       </c>
-      <c r="L13" s="5" t="n">
+      <c r="L13" s="7" t="n">
         <v>0.2115</v>
       </c>
       <c r="M13" t="inlineStr">
@@ -1516,12 +1620,18 @@
       <c r="T13" t="n">
         <v>5</v>
       </c>
-      <c r="U13" t="inlineStr">
+      <c r="U13" s="8" t="n"/>
+      <c r="V13" s="9" t="n"/>
+      <c r="W13" s="9" t="n"/>
+      <c r="X13" s="8" t="n"/>
+      <c r="Y13" s="9" t="n"/>
+      <c r="Z13" s="9" t="n"/>
+      <c r="AB13" t="inlineStr">
         <is>
           <t>1º colocado (Rota Agro Brasil, 19,70%) inabilitado; desconto da Way a verificar</t>
         </is>
       </c>
-      <c r="V13" t="inlineStr">
+      <c r="AC13" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/bndes-cn2-centro-oeste-norte</t>
         </is>
@@ -1556,7 +1666,7 @@
       <c r="F14" t="n">
         <v>30</v>
       </c>
-      <c r="G14" s="2" t="n">
+      <c r="G14" s="6" t="n">
         <v>627.52</v>
       </c>
       <c r="H14" s="3" t="n">
@@ -1568,10 +1678,10 @@
       <c r="J14" s="4" t="n">
         <v>0.1233</v>
       </c>
-      <c r="K14" s="5" t="n">
+      <c r="K14" s="7" t="n">
         <v>0.16788</v>
       </c>
-      <c r="L14" s="5" t="n">
+      <c r="L14" s="7" t="n">
         <v>0.23503</v>
       </c>
       <c r="M14" t="inlineStr">
@@ -1598,12 +1708,18 @@
       <c r="S14" s="4" t="n">
         <v>0.212</v>
       </c>
-      <c r="U14" t="inlineStr">
+      <c r="U14" s="8" t="n"/>
+      <c r="V14" s="9" t="n"/>
+      <c r="W14" s="9" t="n"/>
+      <c r="X14" s="8" t="n"/>
+      <c r="Y14" s="9" t="n"/>
+      <c r="Z14" s="9" t="n"/>
+      <c r="AB14" t="inlineStr">
         <is>
           <t>página escreve '/100 km', mas os valores são por km</t>
         </is>
       </c>
-      <c r="V14" t="inlineStr">
+      <c r="AC14" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-272-369-376-pr-e-pr-182-272-317-323-444-862-897-986</t>
         </is>
@@ -1638,7 +1754,7 @@
       <c r="F15" t="n">
         <v>30</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="G15" s="6" t="n">
         <v>432.7</v>
       </c>
       <c r="H15" s="3" t="n">
@@ -1650,10 +1766,10 @@
       <c r="J15" s="4" t="n">
         <v>0.1233</v>
       </c>
-      <c r="K15" s="5" t="n">
+      <c r="K15" s="7" t="n">
         <v>0.17911</v>
       </c>
-      <c r="L15" s="5" t="n">
+      <c r="L15" s="7" t="n">
         <v>0.25075</v>
       </c>
       <c r="M15" t="inlineStr">
@@ -1677,12 +1793,18 @@
       <c r="S15" s="4" t="n">
         <v>0.24</v>
       </c>
-      <c r="U15" t="inlineStr">
+      <c r="U15" s="8" t="n"/>
+      <c r="V15" s="9" t="n"/>
+      <c r="W15" s="9" t="n"/>
+      <c r="X15" s="8" t="n"/>
+      <c r="Y15" s="9" t="n"/>
+      <c r="Z15" s="9" t="n"/>
+      <c r="AB15" t="inlineStr">
         <is>
           <t>desconto 'quase 24%' (governo do PR); valor exato a verificar</t>
         </is>
       </c>
-      <c r="V15" t="inlineStr">
+      <c r="AC15" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovias-integradas-do-parana-lote-5 ; https://www.parana.pr.gov.br/Audio/Grupo-Patria-arremata-Lote-5-e-investira-R-119-bilhoes-em-novas-obras-no-Parana</t>
         </is>
@@ -1717,7 +1839,7 @@
       <c r="F16" t="n">
         <v>30</v>
       </c>
-      <c r="G16" s="2" t="n">
+      <c r="G16" s="6" t="n">
         <v>530.6</v>
       </c>
       <c r="H16" s="3" t="n">
@@ -1729,10 +1851,10 @@
       <c r="J16" s="4" t="n">
         <v>0.1091</v>
       </c>
-      <c r="K16" s="5" t="n">
+      <c r="K16" s="7" t="n">
         <v>0.13482</v>
       </c>
-      <c r="L16" s="5" t="n">
+      <c r="L16" s="7" t="n">
         <v>0.17527</v>
       </c>
       <c r="M16" t="inlineStr">
@@ -1762,8 +1884,13 @@
       <c r="T16" t="n">
         <v>4</v>
       </c>
-      <c r="U16" t="inlineStr"/>
-      <c r="V16" t="inlineStr">
+      <c r="U16" s="8" t="n"/>
+      <c r="V16" s="9" t="n"/>
+      <c r="W16" s="9" t="n"/>
+      <c r="X16" s="8" t="n"/>
+      <c r="Y16" s="9" t="n"/>
+      <c r="Z16" s="9" t="n"/>
+      <c r="AC16" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovia-br-153-262-go-mg-rota-sertaneja</t>
         </is>
@@ -1795,12 +1922,12 @@
           <t>dez/2025</t>
         </is>
       </c>
-      <c r="G17" s="2" t="n"/>
+      <c r="G17" s="6" t="n"/>
       <c r="H17" s="3" t="n"/>
       <c r="I17" s="3" t="n"/>
       <c r="J17" s="4" t="n"/>
-      <c r="K17" s="5" t="n"/>
-      <c r="L17" s="5" t="n"/>
+      <c r="K17" s="7" t="n"/>
+      <c r="L17" s="7" t="n"/>
       <c r="M17" t="inlineStr">
         <is>
           <t>n/d</t>
@@ -1817,12 +1944,18 @@
         </is>
       </c>
       <c r="S17" s="4" t="n"/>
-      <c r="U17" t="inlineStr">
+      <c r="U17" s="8" t="n"/>
+      <c r="V17" s="9" t="n"/>
+      <c r="W17" s="9" t="n"/>
+      <c r="X17" s="8" t="n"/>
+      <c r="Y17" s="9" t="n"/>
+      <c r="Z17" s="9" t="n"/>
+      <c r="AB17" t="inlineStr">
         <is>
           <t>nova licitação de trecho já concedido; dados a buscar</t>
         </is>
       </c>
-      <c r="V17" t="inlineStr">
+      <c r="AC17" t="inlineStr">
         <is>
           <t>https://agenciainfra.com/blog/motiva-arremata-fernao-dias-e-ministerio-conclui-agenda-de-2025/</t>
         </is>
@@ -1857,7 +1990,7 @@
       <c r="F18" t="n">
         <v>30</v>
       </c>
-      <c r="G18" s="2" t="n">
+      <c r="G18" s="6" t="n">
         <v>734.9</v>
       </c>
       <c r="H18" s="3" t="n">
@@ -1869,10 +2002,10 @@
       <c r="J18" s="4" t="n">
         <v>0.126</v>
       </c>
-      <c r="K18" s="5" t="n">
+      <c r="K18" s="7" t="n">
         <v>0.12644</v>
       </c>
-      <c r="L18" s="5" t="n">
+      <c r="L18" s="7" t="n">
         <v>0.17702</v>
       </c>
       <c r="M18" t="inlineStr">
@@ -1905,12 +2038,35 @@
       <c r="T18" t="n">
         <v>3</v>
       </c>
-      <c r="U18" t="inlineStr">
+      <c r="U18" s="8" t="n">
+        <v>4448</v>
+      </c>
+      <c r="V18" s="9" t="n">
+        <v>0.466</v>
+      </c>
+      <c r="W18" s="9" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="X18" s="8" t="n">
+        <v>42893</v>
+      </c>
+      <c r="Y18" s="9" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="Z18" s="9" t="n">
+        <v>0.21</v>
+      </c>
+      <c r="AA18" t="inlineStr">
+        <is>
+          <t>BNDES/Dynatest, Estudo de Demanda Lote 01 (V10, dez/2025): contagem 2021 (Tab. 10), projeção por praça em veículos equivalentes (Tab. 54) e fuga (Tab. 55), cenário de tarifa R$ 0,20/km</t>
+        </is>
+      </c>
+      <c r="AB18" t="inlineStr">
         <is>
           <t>propostas iniciais: Eco 13,5%, Atlas 13,7%, FIP 0,01%; viva-voz</t>
         </is>
       </c>
-      <c r="V18" t="inlineStr">
+      <c r="AC18" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovias-BR%20116-251-MG ; https://www.gov.br/antt/pt-br/assuntos/ultimas-noticias/ecorodovias-vence-primeiro-leilao-rodoviario-federal-de-2026-com-19-de-desconto-e-assume-735-km-em-minas-gerais</t>
         </is>
@@ -1945,7 +2101,7 @@
       <c r="F19" t="n">
         <v>30</v>
       </c>
-      <c r="G19" s="2" t="n">
+      <c r="G19" s="6" t="n">
         <v>502</v>
       </c>
       <c r="H19" s="3" t="n">
@@ -1957,10 +2113,10 @@
       <c r="J19" s="4" t="n">
         <v>0.1249</v>
       </c>
-      <c r="K19" s="5" t="n">
+      <c r="K19" s="7" t="n">
         <v>0.0953</v>
       </c>
-      <c r="L19" s="5" t="n">
+      <c r="L19" s="7" t="n">
         <v>0.1239</v>
       </c>
       <c r="M19" t="inlineStr">
@@ -1987,12 +2143,18 @@
       <c r="S19" s="4" t="n">
         <v>0.196</v>
       </c>
-      <c r="U19" t="inlineStr">
+      <c r="U19" s="8" t="n"/>
+      <c r="V19" s="9" t="n"/>
+      <c r="W19" s="9" t="n"/>
+      <c r="X19" s="8" t="n"/>
+      <c r="Y19" s="9" t="n"/>
+      <c r="Z19" s="9" t="n"/>
+      <c r="AB19" t="inlineStr">
         <is>
           <t>página escreve '/100 km', mas os valores são por km; nº de propostas a verificar</t>
         </is>
       </c>
-      <c r="V19" t="inlineStr">
+      <c r="AC19" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/BR-116-BA-PE ; https://movimentoeconomico.com.br/estados/bahia/2026/05/28/consorcio-com-odebrecht-e-grupo-chines-vence-leilao-da-rota-dos-sertoes/</t>
         </is>
@@ -2024,12 +2186,12 @@
           <t>12/11/2026</t>
         </is>
       </c>
-      <c r="G20" s="2" t="n"/>
+      <c r="G20" s="6" t="n"/>
       <c r="H20" s="3" t="n"/>
       <c r="I20" s="3" t="n"/>
       <c r="J20" s="4" t="n"/>
-      <c r="K20" s="5" t="n"/>
-      <c r="L20" s="5" t="n"/>
+      <c r="K20" s="7" t="n"/>
+      <c r="L20" s="7" t="n"/>
       <c r="M20" t="inlineStr">
         <is>
           <t>n/d</t>
@@ -2041,12 +2203,18 @@
         </is>
       </c>
       <c r="S20" s="4" t="n"/>
-      <c r="U20" t="inlineStr">
+      <c r="U20" s="8" t="n"/>
+      <c r="V20" s="9" t="n"/>
+      <c r="W20" s="9" t="n"/>
+      <c r="X20" s="8" t="n"/>
+      <c r="Y20" s="9" t="n"/>
+      <c r="Z20" s="9" t="n"/>
+      <c r="AB20" t="inlineStr">
         <is>
           <t>envolve a concessionária atual (Via Brasil); verificar se é contrato novo; capex ~R$ 10,6 bi (imprensa)</t>
         </is>
       </c>
-      <c r="V20" t="inlineStr">
+      <c r="AC20" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/noticias-defeso-eleitoral/br-163-mt-pa-sera-o-proximo-leilao-rodoviario-previsto-pela-antt-em-2026-1</t>
         </is>
@@ -2081,7 +2249,7 @@
       <c r="F21" t="n">
         <v>30</v>
       </c>
-      <c r="G21" s="2" t="n">
+      <c r="G21" s="6" t="n">
         <v>887.6</v>
       </c>
       <c r="H21" s="3" t="n">
@@ -2093,10 +2261,10 @@
       <c r="J21" s="4" t="n">
         <v>0.1107</v>
       </c>
-      <c r="K21" s="5" t="n">
+      <c r="K21" s="7" t="n">
         <v>0.1577</v>
       </c>
-      <c r="L21" s="5" t="n">
+      <c r="L21" s="7" t="n">
         <v>0.205</v>
       </c>
       <c r="M21" t="inlineStr">
@@ -2116,8 +2284,13 @@
         <v>129</v>
       </c>
       <c r="S21" s="4" t="n"/>
-      <c r="U21" t="inlineStr"/>
-      <c r="V21" t="inlineStr">
+      <c r="U21" s="8" t="n"/>
+      <c r="V21" s="9" t="n"/>
+      <c r="W21" s="9" t="n"/>
+      <c r="X21" s="8" t="n"/>
+      <c r="Y21" s="9" t="n"/>
+      <c r="Z21" s="9" t="n"/>
+      <c r="AC21" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/copy_of_rodovias2013contratacao-bndes-6-700m-2013lotes-centro-oeste-e-norte</t>
         </is>
@@ -2152,7 +2325,7 @@
       <c r="F22" t="n">
         <v>30</v>
       </c>
-      <c r="G22" s="2" t="n">
+      <c r="G22" s="6" t="n">
         <v>653.3</v>
       </c>
       <c r="H22" s="3" t="n">
@@ -2164,10 +2337,10 @@
       <c r="J22" s="4" t="n">
         <v>0.1249</v>
       </c>
-      <c r="K22" s="5" t="n">
+      <c r="K22" s="7" t="n">
         <v>0.0839</v>
       </c>
-      <c r="L22" s="5" t="n">
+      <c r="L22" s="7" t="n">
         <v>0.1133</v>
       </c>
       <c r="M22" t="inlineStr">
@@ -2181,12 +2354,18 @@
         </is>
       </c>
       <c r="S22" s="4" t="n"/>
-      <c r="U22" t="inlineStr">
+      <c r="U22" s="8" t="n"/>
+      <c r="V22" s="9" t="n"/>
+      <c r="W22" s="9" t="n"/>
+      <c r="X22" s="8" t="n"/>
+      <c r="Y22" s="9" t="n"/>
+      <c r="Z22" s="9" t="n"/>
+      <c r="AB22" t="inlineStr">
         <is>
           <t>texto cita 663 km</t>
         </is>
       </c>
-      <c r="V22" t="inlineStr">
+      <c r="AC22" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/BR-116-324-BA</t>
         </is>
@@ -2221,7 +2400,7 @@
       <c r="F23" t="n">
         <v>30</v>
       </c>
-      <c r="G23" s="2" t="n">
+      <c r="G23" s="6" t="n">
         <v>232.1</v>
       </c>
       <c r="H23" s="3" t="n">
@@ -2233,10 +2412,10 @@
       <c r="J23" s="4" t="n">
         <v>0.0988</v>
       </c>
-      <c r="K23" s="5" t="n">
+      <c r="K23" s="7" t="n">
         <v>0.15729</v>
       </c>
-      <c r="L23" s="5" t="n"/>
+      <c r="L23" s="7" t="n"/>
       <c r="M23" t="inlineStr">
         <is>
           <t>n/d</t>
@@ -2248,19 +2427,25 @@
         </is>
       </c>
       <c r="S23" s="4" t="n"/>
-      <c r="U23" t="inlineStr">
+      <c r="U23" s="8" t="n"/>
+      <c r="V23" s="9" t="n"/>
+      <c r="W23" s="9" t="n"/>
+      <c r="X23" s="8" t="n"/>
+      <c r="Y23" s="9" t="n"/>
+      <c r="Z23" s="9" t="n"/>
+      <c r="AB23" t="inlineStr">
         <is>
           <t>edital ainda não publicado</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="AC23" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/BR-040-MG-BH-JF</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:V23"/>
+  <autoFilter ref="A1:AC23"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2271,7 +2456,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2326,6 +2511,41 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>vdma_contagem: média do volume diário (veículos) nos postos de contagem do estudo de demanda, nos trechos concedidos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>pct_caminhoes / pct_pesados: participação de caminhões (leves + pesados) e só pesados no volume contado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>vdma_equiv_pracas_ano1: soma do volume diário em veículos EQUIVALENTES (por eixo, que é o que paga) nas praças, no 1º ano do contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cresc_trafego_aa: crescimento médio anual do tráfego equivalente projetado nas praças ao longo do contrato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>fuga_pct: tráfego que desvia para evitar o pedágio, em % do tráfego potencial na praça (cenário de tarifa do estudo).</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Atualiza dados e premissas
</commit_message>
<xml_diff>
--- a/dados/leiloes_rodovias.xlsx
+++ b/dados/leiloes_rodovias.xlsx
@@ -9,6 +9,8 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="leiloes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="notas" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regiao" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="municipios_regiao" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'leiloes'!$A$1:$AC$23</definedName>
@@ -19,11 +21,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="#,##0.0"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.00000"/>
     <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.000"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -63,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -76,6 +79,8 @@
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -681,6 +686,9 @@
       <c r="S2" s="4" t="n">
         <v>0.1825</v>
       </c>
+      <c r="T2" t="n">
+        <v>2</v>
+      </c>
       <c r="U2" s="8" t="n"/>
       <c r="V2" s="9" t="n"/>
       <c r="W2" s="9" t="n"/>
@@ -689,7 +697,7 @@
       <c r="Z2" s="9" t="n"/>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>EPR ofereceu 8,30%; nº total de propostas a verificar</t>
+          <t>2 propostas: Pátria 18,25% e Infraestrutura PR 8,30%</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -951,12 +959,12 @@
       <c r="Z5" s="9" t="n"/>
       <c r="AB5" t="inlineStr">
         <is>
-          <t>desconto a verificar (critério inclui outorga)</t>
+          <t>4 propostas; BTG Pactual perdeu com 7,5%; desconto da Vinci a verificar (critério inclui outorga)</t>
         </is>
       </c>
       <c r="AC5" t="inlineStr">
         <is>
-          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-040-go-mg-rota-dos-cristais</t>
+          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-040-go-mg-rota-dos-cristais ; https://blogs.correiobraziliense.com.br/capital-sa/2024/09/26/empresa-francesa-ganha-concessao-da-rota-dos-cristais/</t>
         </is>
       </c>
     </row>
@@ -1019,11 +1027,14 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>Rotas do Brasil</t>
+          <t>Rotas do Brasil (Kinea + Way Brasil)</t>
         </is>
       </c>
       <c r="S6" s="4" t="n">
         <v>0.153</v>
+      </c>
+      <c r="T6" t="n">
+        <v>2</v>
       </c>
       <c r="U6" s="8" t="n"/>
       <c r="V6" s="9" t="n"/>
@@ -1031,9 +1042,14 @@
       <c r="X6" s="8" t="n"/>
       <c r="Y6" s="9" t="n"/>
       <c r="Z6" s="9" t="n"/>
+      <c r="AB6" t="inlineStr">
+        <is>
+          <t>KINEA no consórcio vencedor; 2 propostas, decidido no viva-voz: Rotas do Brasil 15,3% vs. BTG Pactual Infraestrutura III 15,2%; relicitação da Concebra</t>
+        </is>
+      </c>
       <c r="AC6" t="inlineStr">
         <is>
-          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovia-br-262-mg-rota-do-zebu</t>
+          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovia-br-262-mg-rota-do-zebu ; https://jornaldebrasilia.com.br/noticias/economia/gestora-kinea-leva-rota-do-zebu-em-mg-e-consolida-participacao-de-fundos-em-leiloes/</t>
         </is>
       </c>
     </row>
@@ -1111,12 +1127,27 @@
       <c r="T7" t="n">
         <v>4</v>
       </c>
-      <c r="U7" s="8" t="n"/>
-      <c r="V7" s="9" t="n"/>
-      <c r="W7" s="9" t="n"/>
-      <c r="X7" s="8" t="n"/>
-      <c r="Y7" s="9" t="n"/>
+      <c r="U7" s="8" t="n">
+        <v>8280</v>
+      </c>
+      <c r="V7" s="9" t="n">
+        <v>0.43</v>
+      </c>
+      <c r="W7" s="9" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="X7" s="8" t="n">
+        <v>138500</v>
+      </c>
+      <c r="Y7" s="9" t="n">
+        <v>0.024</v>
+      </c>
       <c r="Z7" s="9" t="n"/>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>Engimind/IFC, Estudo de Tráfego Lote 3, Tomos I e II (set/2021). Valores por praça LIDOS DOS GRÁFICOS da Tabela 5 do Tomo II (ano 2023, 7 praças), precisão de ~10%; 'pesados' = 4 ou mais eixos; crescimento do tráfego equivalente estimado nas praças de Witmarsum e Tibagi; impacto da ferrovia (Nova Ferroeste) de −2% a −3% nas praças do lote (Tab. 123 do Tomo I)</t>
+        </is>
+      </c>
       <c r="AC7" t="inlineStr">
         <is>
           <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-369-373-376-pr-e-pr-090-170-323-445</t>
@@ -1371,12 +1402,27 @@
       <c r="T10" t="n">
         <v>1</v>
       </c>
-      <c r="U10" s="8" t="n"/>
-      <c r="V10" s="9" t="n"/>
-      <c r="W10" s="9" t="n"/>
+      <c r="U10" s="8" t="n">
+        <v>6072</v>
+      </c>
+      <c r="V10" s="9" t="n">
+        <v>0.356</v>
+      </c>
+      <c r="W10" s="9" t="n">
+        <v>0.224</v>
+      </c>
       <c r="X10" s="8" t="n"/>
       <c r="Y10" s="9" t="n"/>
-      <c r="Z10" s="9" t="n"/>
+      <c r="Z10" s="9" t="inlineStr">
+        <is>
+          <t>baixa (estudo: sem troca expressiva de caminhos)</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>BNDES/Consórcio (LOGIT), Lote CN5, Tomos I e IIb, 2021-2023; contagem: média de 10 pontos na BR-364/RO, sem motos e ônibus; receita ano 2 R$ 366 mi a R$ 0,12/km</t>
+        </is>
+      </c>
       <c r="AB10" t="inlineStr">
         <is>
           <t>NeoFeed: 'apenas um concorrente'</t>
@@ -1706,7 +1752,7 @@
         </is>
       </c>
       <c r="S14" s="4" t="n">
-        <v>0.212</v>
+        <v>0.213</v>
       </c>
       <c r="U14" s="8" t="n"/>
       <c r="V14" s="9" t="n"/>
@@ -1716,12 +1762,12 @@
       <c r="Z14" s="9" t="n"/>
       <c r="AB14" t="inlineStr">
         <is>
-          <t>página escreve '/100 km', mas os valores são por km</t>
+          <t>ANTT informa 21,20%; Diário do Transporte informa 21,30% (usado o da imprensa, a confirmar na ata); nº de propostas a verificar</t>
         </is>
       </c>
       <c r="AC14" t="inlineStr">
         <is>
-          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-272-369-376-pr-e-pr-182-272-317-323-444-862-897-986</t>
+          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/br-272-369-376-pr-e-pr-182-272-317-323-444-862-897-986 ; https://diariodotransporte.com.br/2025/10/23/epr-vence-leilao-do-lote-4-das-rodovias-integradas-do-parana/</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1837,7 @@
         </is>
       </c>
       <c r="S15" s="4" t="n">
-        <v>0.24</v>
+        <v>0.2383</v>
       </c>
       <c r="U15" s="8" t="n"/>
       <c r="V15" s="9" t="n"/>
@@ -1801,12 +1847,12 @@
       <c r="Z15" s="9" t="n"/>
       <c r="AB15" t="inlineStr">
         <is>
-          <t>desconto 'quase 24%' (governo do PR); valor exato a verificar</t>
+          <t>vencedora Reúne Rodovias Holding II (Pátria), 23,83% + aporte de R$ 399,5 mi; nº de propostas a verificar</t>
         </is>
       </c>
       <c r="AC15" t="inlineStr">
         <is>
-          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovias-integradas-do-parana-lote-5 ; https://www.parana.pr.gov.br/Audio/Grupo-Patria-arremata-Lote-5-e-investira-R-119-bilhoes-em-novas-obras-no-Parana</t>
+          <t>https://www.gov.br/antt/pt-br/assuntos/rodovias/novos-projetos-em-rodovias/rodovias-integradas-do-parana-lote-5 ; https://www.parana.pr.gov.br/Audio/Grupo-Patria-arremata-Lote-5-e-investira-R-119-bilhoes-em-novas-obras-no-Parana ; https://diariodotransporte.com.br/2025/10/30/reune-rodovias-holding-ii-s-a-e-a-vencedora-do-leilao-do-lote-5-de-rodovias-integradas-do-parana/</t>
         </is>
       </c>
     </row>
@@ -2354,12 +2400,25 @@
         </is>
       </c>
       <c r="S22" s="4" t="n"/>
-      <c r="U22" s="8" t="n"/>
-      <c r="V22" s="9" t="n"/>
-      <c r="W22" s="9" t="n"/>
+      <c r="U22" s="8" t="n">
+        <v>13742</v>
+      </c>
+      <c r="V22" s="9" t="n">
+        <v>0.421</v>
+      </c>
+      <c r="W22" s="9" t="n">
+        <v>0.238</v>
+      </c>
       <c r="X22" s="8" t="n"/>
-      <c r="Y22" s="9" t="n"/>
+      <c r="Y22" s="9" t="n">
+        <v>0.016</v>
+      </c>
       <c r="Z22" s="9" t="n"/>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>Consórcio EVTEA/Infra S.A., Estudo de Tráfego Rota 2 de Julho (mai/2026): contagem 2022 em 10 pontos (Tab. 18-20); crescimento 1,77% a.a. leves e 1,45% a.a. comerciais em 2025-2060 (Tab. 30). Média puxada pela BR-324 perto de Salvador (~29 mil leves/dia); sem a BR-324, os caminhões são ~57% do volume</t>
+        </is>
+      </c>
       <c r="AB22" t="inlineStr">
         <is>
           <t>texto cita 663 km</t>
@@ -2456,7 +2515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="140" customWidth="1" min="1" max="1"/>
@@ -2546,6 +2605,4115 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Atenção: as categorias de caminhão variam entre estudos (cam. leve/pesado; comerciais leves/pesados; pesados 2-3 eixos / 4+ eixos). Comparar pct_pesados com cautela.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>ABA regiao — fonte: IBGE, PIB dos Municípios, base 2010-2023 (baixada em 23/10/2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>PIB e PIB per capita: 2023. Composição setorial (pct_*): 2021, último ano com abertura por setor na base (2022-2023 só têm o PIB total).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>pct_* = parcela do valor adicionado bruto (VAB, sem impostos); serviços exclui administração pública.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>hhi_setorial = soma dos quadrados das 4 parcelas; quanto maior, mais concentrada a economia. Mede pouco aqui porque serviços domina em todos.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>pct_munic_adm_publica_principal = fração dos municípios do lote cuja maior atividade é administração pública (sinal de economia pobre e dependente de transferências).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>populacao = PIB / PIB per capita (estimativa IBGE embutida no cálculo do per capita).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Listas de municípios: Rota das Gerais vem do estudo de demanda; as demais foram montadas pelo traçado e precisam ser conferidas no PER de cada lote.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="19" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="17" customWidth="1" min="13" max="13"/>
+    <col width="25" customWidth="1" min="14" max="14"/>
+    <col width="33" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>leilao</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>n_propostas</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>desconto</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>n_municipios</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>populacao_mil</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>pib_bi</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>pib_per_capita</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>pct_agro</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>pct_industria</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>pct_servicos</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>pct_adm_publica</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>hhi_setorial</t>
+        </is>
+      </c>
+      <c r="M1" s="10" t="inlineStr">
+        <is>
+          <t>maior_municipio</t>
+        </is>
+      </c>
+      <c r="N1" s="10" t="inlineStr">
+        <is>
+          <t>pct_pib_maior_municipio</t>
+        </is>
+      </c>
+      <c r="O1" s="10" t="inlineStr">
+        <is>
+          <t>pct_munic_adm_publica_principal</t>
+        </is>
+      </c>
+      <c r="P1" s="10" t="inlineStr">
+        <is>
+          <t>status_lista</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3</v>
+      </c>
+      <c r="C2" s="9" t="n">
+        <v>0.19</v>
+      </c>
+      <c r="D2" t="n">
+        <v>30</v>
+      </c>
+      <c r="E2" s="8" t="n">
+        <v>1152.60601260907</v>
+      </c>
+      <c r="F2" s="6" t="n">
+        <v>32.64662292300001</v>
+      </c>
+      <c r="G2" s="8" t="n">
+        <v>28324.18238830824</v>
+      </c>
+      <c r="H2" s="9" t="n">
+        <v>0.0399277367978342</v>
+      </c>
+      <c r="I2" s="9" t="n">
+        <v>0.179462511259183</v>
+      </c>
+      <c r="J2" s="9" t="n">
+        <v>0.5421915875100943</v>
+      </c>
+      <c r="K2" s="9" t="n">
+        <v>0.2384181644328884</v>
+      </c>
+      <c r="L2" s="11" t="n">
+        <v>0.3846159558115136</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>Montes Claros</t>
+        </is>
+      </c>
+      <c r="N2" s="9" t="n">
+        <v>0.4081965425162391</v>
+      </c>
+      <c r="O2" s="9" t="n">
+        <v>0.6666666666666666</v>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>lista do estudo de demanda (Tabela 4)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4</v>
+      </c>
+      <c r="C3" s="9" t="n">
+        <v>0.266</v>
+      </c>
+      <c r="D3" t="n">
+        <v>20</v>
+      </c>
+      <c r="E3" s="8" t="n">
+        <v>1554.67802106522</v>
+      </c>
+      <c r="F3" s="6" t="n">
+        <v>91.14624823299999</v>
+      </c>
+      <c r="G3" s="8" t="n">
+        <v>58627.08998133854</v>
+      </c>
+      <c r="H3" s="9" t="n">
+        <v>0.08050268426000121</v>
+      </c>
+      <c r="I3" s="9" t="n">
+        <v>0.2947746516145089</v>
+      </c>
+      <c r="J3" s="9" t="n">
+        <v>0.5005543011334007</v>
+      </c>
+      <c r="K3" s="9" t="n">
+        <v>0.124168362992089</v>
+      </c>
+      <c r="L3" s="11" t="n">
+        <v>0.3593451681588029</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="N3" s="9" t="n">
+        <v>0.3071935260288927</v>
+      </c>
+      <c r="O3" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>aproximada pelo traçado (a conferir no PER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr"/>
+      <c r="D4" t="n">
+        <v>17</v>
+      </c>
+      <c r="E4" s="8" t="n">
+        <v>4068.328966326889</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>135.166970275</v>
+      </c>
+      <c r="G4" s="8" t="n">
+        <v>33224.19877885051</v>
+      </c>
+      <c r="H4" s="9" t="n">
+        <v>0.0081918527573427</v>
+      </c>
+      <c r="I4" s="9" t="n">
+        <v>0.1929766829647669</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>0.6359147474252045</v>
+      </c>
+      <c r="K4" s="9" t="n">
+        <v>0.1629167168526859</v>
+      </c>
+      <c r="L4" s="11" t="n">
+        <v>0.468236529242602</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="N4" s="9" t="n">
+        <v>0.5674372745202083</v>
+      </c>
+      <c r="O4" s="9" t="n">
+        <v>0.4117647058823529</v>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>aproximada pelo traçado (a conferir no PER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" s="9" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="D5" t="n">
+        <v>11</v>
+      </c>
+      <c r="E5" s="8" t="n">
+        <v>1035.217986671698</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>52.60816425200001</v>
+      </c>
+      <c r="G5" s="8" t="n">
+        <v>50818.44107166178</v>
+      </c>
+      <c r="H5" s="9" t="n">
+        <v>0.1083563251742534</v>
+      </c>
+      <c r="I5" s="9" t="n">
+        <v>0.1968461876234508</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0.45218402384294</v>
+      </c>
+      <c r="K5" s="9" t="n">
+        <v>0.2426134633593556</v>
+      </c>
+      <c r="L5" s="11" t="n">
+        <v>0.3138211988091692</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Porto Velho</t>
+        </is>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>0.4828564880599171</v>
+      </c>
+      <c r="O5" s="9" t="n">
+        <v>0.2727272727272727</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>aproximada pelo traçado (a conferir no PER)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Brasil (referência)</t>
+        </is>
+      </c>
+      <c r="C6" s="9" t="inlineStr"/>
+      <c r="D6" t="n">
+        <v>5570</v>
+      </c>
+      <c r="E6" s="8" t="n">
+        <v>203080.7568428575</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>10943.34543888</v>
+      </c>
+      <c r="G6" s="8" t="n">
+        <v>53886.66857957342</v>
+      </c>
+      <c r="H6" s="9" t="n">
+        <v>0.0766249775234723</v>
+      </c>
+      <c r="I6" s="9" t="n">
+        <v>0.2584650322115907</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>0.5068913024224839</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>0.158018687842453</v>
+      </c>
+      <c r="L6" s="11" t="n">
+        <v>0.3545842582356239</v>
+      </c>
+      <c r="N6" s="9" t="inlineStr"/>
+      <c r="O6" s="9" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>todos os municípios</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:L79"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="40" customWidth="1" min="12" max="12"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="10" t="inlineStr">
+        <is>
+          <t>leilao</t>
+        </is>
+      </c>
+      <c r="B1" s="10" t="inlineStr">
+        <is>
+          <t>municipio</t>
+        </is>
+      </c>
+      <c r="C1" s="10" t="inlineStr">
+        <is>
+          <t>uf</t>
+        </is>
+      </c>
+      <c r="D1" s="10" t="inlineStr">
+        <is>
+          <t>codigo_ibge</t>
+        </is>
+      </c>
+      <c r="E1" s="10" t="inlineStr">
+        <is>
+          <t>populacao</t>
+        </is>
+      </c>
+      <c r="F1" s="10" t="inlineStr">
+        <is>
+          <t>pib_mil</t>
+        </is>
+      </c>
+      <c r="G1" s="10" t="inlineStr">
+        <is>
+          <t>pib_per_capita</t>
+        </is>
+      </c>
+      <c r="H1" s="10" t="inlineStr">
+        <is>
+          <t>va_agro</t>
+        </is>
+      </c>
+      <c r="I1" s="10" t="inlineStr">
+        <is>
+          <t>va_industria</t>
+        </is>
+      </c>
+      <c r="J1" s="10" t="inlineStr">
+        <is>
+          <t>va_servicos</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>va_adm_publica</t>
+        </is>
+      </c>
+      <c r="L1" s="10" t="inlineStr">
+        <is>
+          <t>atividade_principal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Águas Vermelhas</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>3101003</v>
+      </c>
+      <c r="E2" t="n">
+        <v>14037</v>
+      </c>
+      <c r="F2" t="n">
+        <v>278389.902</v>
+      </c>
+      <c r="G2" t="n">
+        <v>19832.58</v>
+      </c>
+      <c r="H2" t="n">
+        <v>52991.442</v>
+      </c>
+      <c r="I2" t="n">
+        <v>8903.823</v>
+      </c>
+      <c r="J2" t="n">
+        <v>88300.49000000001</v>
+      </c>
+      <c r="K2" t="n">
+        <v>65954.424</v>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Cachoeira de Pajeú</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D3" t="n">
+        <v>3102704</v>
+      </c>
+      <c r="E3" t="n">
+        <v>9110</v>
+      </c>
+      <c r="F3" t="n">
+        <v>146445.066</v>
+      </c>
+      <c r="G3" t="n">
+        <v>16075.2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>7112.874</v>
+      </c>
+      <c r="I3" t="n">
+        <v>4003.348</v>
+      </c>
+      <c r="J3" t="n">
+        <v>57452.326</v>
+      </c>
+      <c r="K3" t="n">
+        <v>45896.879</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Campanário</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D4" t="n">
+        <v>3110806</v>
+      </c>
+      <c r="E4" t="n">
+        <v>2923</v>
+      </c>
+      <c r="F4" t="n">
+        <v>61166.633</v>
+      </c>
+      <c r="G4" t="n">
+        <v>20925.98</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6982.226</v>
+      </c>
+      <c r="I4" t="n">
+        <v>1858.495</v>
+      </c>
+      <c r="J4" t="n">
+        <v>18931.903</v>
+      </c>
+      <c r="K4" t="n">
+        <v>23141.669</v>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Caraí</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D5" t="n">
+        <v>3113008</v>
+      </c>
+      <c r="E5" t="n">
+        <v>19548</v>
+      </c>
+      <c r="F5" t="n">
+        <v>273822.674</v>
+      </c>
+      <c r="G5" t="n">
+        <v>14007.71</v>
+      </c>
+      <c r="H5" t="n">
+        <v>22223.454</v>
+      </c>
+      <c r="I5" t="n">
+        <v>22098.152</v>
+      </c>
+      <c r="J5" t="n">
+        <v>51314.401</v>
+      </c>
+      <c r="K5" t="n">
+        <v>103732.462</v>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Catuji</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D6" t="n">
+        <v>3115458</v>
+      </c>
+      <c r="E6" t="n">
+        <v>7030</v>
+      </c>
+      <c r="F6" t="n">
+        <v>109879.753</v>
+      </c>
+      <c r="G6" t="n">
+        <v>15630.12</v>
+      </c>
+      <c r="H6" t="n">
+        <v>5941.277</v>
+      </c>
+      <c r="I6" t="n">
+        <v>1973.977</v>
+      </c>
+      <c r="J6" t="n">
+        <v>32998.783</v>
+      </c>
+      <c r="K6" t="n">
+        <v>36113.22</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Curral de Dentro</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D7" t="n">
+        <v>3120870</v>
+      </c>
+      <c r="E7" t="n">
+        <v>7406</v>
+      </c>
+      <c r="F7" t="n">
+        <v>94746.856</v>
+      </c>
+      <c r="G7" t="n">
+        <v>12793.26</v>
+      </c>
+      <c r="H7" t="n">
+        <v>10329.345</v>
+      </c>
+      <c r="I7" t="n">
+        <v>4652.813</v>
+      </c>
+      <c r="J7" t="n">
+        <v>22117.166</v>
+      </c>
+      <c r="K7" t="n">
+        <v>39993.202</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Divisa Alegre</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>3122355</v>
+      </c>
+      <c r="E8" t="n">
+        <v>6321</v>
+      </c>
+      <c r="F8" t="n">
+        <v>216685.656</v>
+      </c>
+      <c r="G8" t="n">
+        <v>34280.28</v>
+      </c>
+      <c r="H8" t="n">
+        <v>2845.721</v>
+      </c>
+      <c r="I8" t="n">
+        <v>35775.735</v>
+      </c>
+      <c r="J8" t="n">
+        <v>72726.648</v>
+      </c>
+      <c r="K8" t="n">
+        <v>39502.817</v>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Francisco Sá</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>3126703</v>
+      </c>
+      <c r="E9" t="n">
+        <v>23476</v>
+      </c>
+      <c r="F9" t="n">
+        <v>532917.976</v>
+      </c>
+      <c r="G9" t="n">
+        <v>22700.54</v>
+      </c>
+      <c r="H9" t="n">
+        <v>44167.178</v>
+      </c>
+      <c r="I9" t="n">
+        <v>15791.409</v>
+      </c>
+      <c r="J9" t="n">
+        <v>214235.46</v>
+      </c>
+      <c r="K9" t="n">
+        <v>122379.336</v>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Frei Gaspar</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>3126802</v>
+      </c>
+      <c r="E10" t="n">
+        <v>5640</v>
+      </c>
+      <c r="F10" t="n">
+        <v>91083.395</v>
+      </c>
+      <c r="G10" t="n">
+        <v>16149.54</v>
+      </c>
+      <c r="H10" t="n">
+        <v>23887.096</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2450.859</v>
+      </c>
+      <c r="J10" t="n">
+        <v>18620.726</v>
+      </c>
+      <c r="K10" t="n">
+        <v>32379.315</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Frei Inocêncio</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3126901</v>
+      </c>
+      <c r="E11" t="n">
+        <v>8226</v>
+      </c>
+      <c r="F11" t="n">
+        <v>173509.214</v>
+      </c>
+      <c r="G11" t="n">
+        <v>21092.78</v>
+      </c>
+      <c r="H11" t="n">
+        <v>12081.31</v>
+      </c>
+      <c r="I11" t="n">
+        <v>23500.264</v>
+      </c>
+      <c r="J11" t="n">
+        <v>58643.043</v>
+      </c>
+      <c r="K11" t="n">
+        <v>45352.592</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Fruta de Leite</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>3127073</v>
+      </c>
+      <c r="E12" t="n">
+        <v>4647</v>
+      </c>
+      <c r="F12" t="n">
+        <v>57436.617</v>
+      </c>
+      <c r="G12" t="n">
+        <v>12359.93</v>
+      </c>
+      <c r="H12" t="n">
+        <v>3577.059</v>
+      </c>
+      <c r="I12" t="n">
+        <v>1956.618</v>
+      </c>
+      <c r="J12" t="n">
+        <v>11413.683</v>
+      </c>
+      <c r="K12" t="n">
+        <v>28613.664</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Governador Valadares</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>3127701</v>
+      </c>
+      <c r="E13" t="n">
+        <v>257171</v>
+      </c>
+      <c r="F13" t="n">
+        <v>8612265.515000001</v>
+      </c>
+      <c r="G13" t="n">
+        <v>33488.48</v>
+      </c>
+      <c r="H13" t="n">
+        <v>65862.53200000001</v>
+      </c>
+      <c r="I13" t="n">
+        <v>848298.149</v>
+      </c>
+      <c r="J13" t="n">
+        <v>4130148.099</v>
+      </c>
+      <c r="K13" t="n">
+        <v>1481769.877</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Grão Mogol</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3127800</v>
+      </c>
+      <c r="E14" t="n">
+        <v>13901</v>
+      </c>
+      <c r="F14" t="n">
+        <v>817459.322</v>
+      </c>
+      <c r="G14" t="n">
+        <v>58805.79</v>
+      </c>
+      <c r="H14" t="n">
+        <v>184815.8</v>
+      </c>
+      <c r="I14" t="n">
+        <v>437027.997</v>
+      </c>
+      <c r="J14" t="n">
+        <v>56573.9</v>
+      </c>
+      <c r="K14" t="n">
+        <v>81710.935</v>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>Eletricidade e gás, água, esgoto, atividades de gestão de resíduos e descontaminação</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Itambacuri</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3132701</v>
+      </c>
+      <c r="E15" t="n">
+        <v>21042</v>
+      </c>
+      <c r="F15" t="n">
+        <v>415054.966</v>
+      </c>
+      <c r="G15" t="n">
+        <v>19725.07</v>
+      </c>
+      <c r="H15" t="n">
+        <v>42929.163</v>
+      </c>
+      <c r="I15" t="n">
+        <v>23653.736</v>
+      </c>
+      <c r="J15" t="n">
+        <v>141212.149</v>
+      </c>
+      <c r="K15" t="n">
+        <v>107633.138</v>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Itaobim</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>3133303</v>
+      </c>
+      <c r="E16" t="n">
+        <v>19151</v>
+      </c>
+      <c r="F16" t="n">
+        <v>375951.855</v>
+      </c>
+      <c r="G16" t="n">
+        <v>19630.93</v>
+      </c>
+      <c r="H16" t="n">
+        <v>8640.798000000001</v>
+      </c>
+      <c r="I16" t="n">
+        <v>15744.541</v>
+      </c>
+      <c r="J16" t="n">
+        <v>154032.853</v>
+      </c>
+      <c r="K16" t="n">
+        <v>102688.855</v>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Jampruca</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>3135076</v>
+      </c>
+      <c r="E17" t="n">
+        <v>4296</v>
+      </c>
+      <c r="F17" t="n">
+        <v>84853.38099999999</v>
+      </c>
+      <c r="G17" t="n">
+        <v>19751.72</v>
+      </c>
+      <c r="H17" t="n">
+        <v>30171.757</v>
+      </c>
+      <c r="I17" t="n">
+        <v>5190.581</v>
+      </c>
+      <c r="J17" t="n">
+        <v>16636.74</v>
+      </c>
+      <c r="K17" t="n">
+        <v>28119.167</v>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Medina</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D18" t="n">
+        <v>3141405</v>
+      </c>
+      <c r="E18" t="n">
+        <v>20156</v>
+      </c>
+      <c r="F18" t="n">
+        <v>330715.354</v>
+      </c>
+      <c r="G18" t="n">
+        <v>16407.79</v>
+      </c>
+      <c r="H18" t="n">
+        <v>15763.244</v>
+      </c>
+      <c r="I18" t="n">
+        <v>28655.057</v>
+      </c>
+      <c r="J18" t="n">
+        <v>97836.395</v>
+      </c>
+      <c r="K18" t="n">
+        <v>96274.686</v>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Montes Claros</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D19" t="n">
+        <v>3143302</v>
+      </c>
+      <c r="E19" t="n">
+        <v>414240</v>
+      </c>
+      <c r="F19" t="n">
+        <v>13326238.602</v>
+      </c>
+      <c r="G19" t="n">
+        <v>32170.33</v>
+      </c>
+      <c r="H19" t="n">
+        <v>156030.836</v>
+      </c>
+      <c r="I19" t="n">
+        <v>1961020.907</v>
+      </c>
+      <c r="J19" t="n">
+        <v>5465743.037</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1879776.235</v>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Novorizonte</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D20" t="n">
+        <v>3145372</v>
+      </c>
+      <c r="E20" t="n">
+        <v>4571</v>
+      </c>
+      <c r="F20" t="n">
+        <v>92593.548</v>
+      </c>
+      <c r="G20" t="n">
+        <v>20256.74</v>
+      </c>
+      <c r="H20" t="n">
+        <v>2932.388</v>
+      </c>
+      <c r="I20" t="n">
+        <v>11901.349</v>
+      </c>
+      <c r="J20" t="n">
+        <v>17508.265</v>
+      </c>
+      <c r="K20" t="n">
+        <v>30316.264</v>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Padre Carvalho</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D21" t="n">
+        <v>3146255</v>
+      </c>
+      <c r="E21" t="n">
+        <v>5058</v>
+      </c>
+      <c r="F21" t="n">
+        <v>68448.34600000001</v>
+      </c>
+      <c r="G21" t="n">
+        <v>13532.69</v>
+      </c>
+      <c r="H21" t="n">
+        <v>1181.657</v>
+      </c>
+      <c r="I21" t="n">
+        <v>1599.638</v>
+      </c>
+      <c r="J21" t="n">
+        <v>19492.125</v>
+      </c>
+      <c r="K21" t="n">
+        <v>32659.926</v>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Padre Paraíso</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D22" t="n">
+        <v>3146305</v>
+      </c>
+      <c r="E22" t="n">
+        <v>17334</v>
+      </c>
+      <c r="F22" t="n">
+        <v>254680.841</v>
+      </c>
+      <c r="G22" t="n">
+        <v>14692.56</v>
+      </c>
+      <c r="H22" t="n">
+        <v>7323.528</v>
+      </c>
+      <c r="I22" t="n">
+        <v>13429.014</v>
+      </c>
+      <c r="J22" t="n">
+        <v>86282.697</v>
+      </c>
+      <c r="K22" t="n">
+        <v>94611.777</v>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Pedra Azul</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D23" t="n">
+        <v>3148707</v>
+      </c>
+      <c r="E23" t="n">
+        <v>24410</v>
+      </c>
+      <c r="F23" t="n">
+        <v>428870.193</v>
+      </c>
+      <c r="G23" t="n">
+        <v>17569.45</v>
+      </c>
+      <c r="H23" t="n">
+        <v>14186.543</v>
+      </c>
+      <c r="I23" t="n">
+        <v>108936.95</v>
+      </c>
+      <c r="J23" t="n">
+        <v>136675.201</v>
+      </c>
+      <c r="K23" t="n">
+        <v>121361.357</v>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Ponto dos Volantes</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D24" t="n">
+        <v>3152170</v>
+      </c>
+      <c r="E24" t="n">
+        <v>10883</v>
+      </c>
+      <c r="F24" t="n">
+        <v>149416.361</v>
+      </c>
+      <c r="G24" t="n">
+        <v>13729.34</v>
+      </c>
+      <c r="H24" t="n">
+        <v>9882.455</v>
+      </c>
+      <c r="I24" t="n">
+        <v>4674.395</v>
+      </c>
+      <c r="J24" t="n">
+        <v>40364.353</v>
+      </c>
+      <c r="K24" t="n">
+        <v>60478.333</v>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Riacho dos Machados</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D25" t="n">
+        <v>3154507</v>
+      </c>
+      <c r="E25" t="n">
+        <v>8756</v>
+      </c>
+      <c r="F25" t="n">
+        <v>301729.817</v>
+      </c>
+      <c r="G25" t="n">
+        <v>34459.78</v>
+      </c>
+      <c r="H25" t="n">
+        <v>47609.484</v>
+      </c>
+      <c r="I25" t="n">
+        <v>322182.498</v>
+      </c>
+      <c r="J25" t="n">
+        <v>84269.72900000001</v>
+      </c>
+      <c r="K25" t="n">
+        <v>53552.674</v>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>Indústrias extrativas</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Rubelita</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D26" t="n">
+        <v>3156502</v>
+      </c>
+      <c r="E26" t="n">
+        <v>5679</v>
+      </c>
+      <c r="F26" t="n">
+        <v>85774.927</v>
+      </c>
+      <c r="G26" t="n">
+        <v>15103.88</v>
+      </c>
+      <c r="H26" t="n">
+        <v>10701.716</v>
+      </c>
+      <c r="I26" t="n">
+        <v>15602.703</v>
+      </c>
+      <c r="J26" t="n">
+        <v>17740.777</v>
+      </c>
+      <c r="K26" t="n">
+        <v>33630.229</v>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Salinas</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D27" t="n">
+        <v>3157005</v>
+      </c>
+      <c r="E27" t="n">
+        <v>40178</v>
+      </c>
+      <c r="F27" t="n">
+        <v>903694.482</v>
+      </c>
+      <c r="G27" t="n">
+        <v>22492.27</v>
+      </c>
+      <c r="H27" t="n">
+        <v>27608.563</v>
+      </c>
+      <c r="I27" t="n">
+        <v>62009.728</v>
+      </c>
+      <c r="J27" t="n">
+        <v>317353.958</v>
+      </c>
+      <c r="K27" t="n">
+        <v>197668.723</v>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Santa Cruz de Salinas</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D28" t="n">
+        <v>3157377</v>
+      </c>
+      <c r="E28" t="n">
+        <v>3910</v>
+      </c>
+      <c r="F28" t="n">
+        <v>59169.054</v>
+      </c>
+      <c r="G28" t="n">
+        <v>15132.75</v>
+      </c>
+      <c r="H28" t="n">
+        <v>4873.597</v>
+      </c>
+      <c r="I28" t="n">
+        <v>1057.09</v>
+      </c>
+      <c r="J28" t="n">
+        <v>15787.668</v>
+      </c>
+      <c r="K28" t="n">
+        <v>24646.659</v>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Taiobeiras</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D29" t="n">
+        <v>3168002</v>
+      </c>
+      <c r="E29" t="n">
+        <v>33050</v>
+      </c>
+      <c r="F29" t="n">
+        <v>705372.64</v>
+      </c>
+      <c r="G29" t="n">
+        <v>21342.59</v>
+      </c>
+      <c r="H29" t="n">
+        <v>59332.219</v>
+      </c>
+      <c r="I29" t="n">
+        <v>42629.54</v>
+      </c>
+      <c r="J29" t="n">
+        <v>251983.675</v>
+      </c>
+      <c r="K29" t="n">
+        <v>163118.522</v>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Teófilo Otoni</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D30" t="n">
+        <v>3168606</v>
+      </c>
+      <c r="E30" t="n">
+        <v>137418</v>
+      </c>
+      <c r="F30" t="n">
+        <v>3540247.727</v>
+      </c>
+      <c r="G30" t="n">
+        <v>25762.62</v>
+      </c>
+      <c r="H30" t="n">
+        <v>90726.94899999999</v>
+      </c>
+      <c r="I30" t="n">
+        <v>368265.853</v>
+      </c>
+      <c r="J30" t="n">
+        <v>1572586.047</v>
+      </c>
+      <c r="K30" t="n">
+        <v>647157.249</v>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Rota das Gerais</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Mathias Lobato</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>MG</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>3171501</v>
+      </c>
+      <c r="E31" t="n">
+        <v>3038</v>
+      </c>
+      <c r="F31" t="n">
+        <v>58002.25</v>
+      </c>
+      <c r="G31" t="n">
+        <v>19092.25</v>
+      </c>
+      <c r="H31" t="n">
+        <v>5449.615</v>
+      </c>
+      <c r="I31" t="n">
+        <v>1681.902</v>
+      </c>
+      <c r="J31" t="n">
+        <v>13791.93</v>
+      </c>
+      <c r="K31" t="n">
+        <v>20606.437</v>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Apucarana</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4101408</v>
+      </c>
+      <c r="E32" t="n">
+        <v>130134</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4834012.856</v>
+      </c>
+      <c r="G32" t="n">
+        <v>37146.42</v>
+      </c>
+      <c r="H32" t="n">
+        <v>281831.223</v>
+      </c>
+      <c r="I32" t="n">
+        <v>834984.803</v>
+      </c>
+      <c r="J32" t="n">
+        <v>1691674.371</v>
+      </c>
+      <c r="K32" t="n">
+        <v>647972.165</v>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Arapongas</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>4101507</v>
+      </c>
+      <c r="E33" t="n">
+        <v>119138</v>
+      </c>
+      <c r="F33" t="n">
+        <v>5715471.043</v>
+      </c>
+      <c r="G33" t="n">
+        <v>47973.54</v>
+      </c>
+      <c r="H33" t="n">
+        <v>373977.951</v>
+      </c>
+      <c r="I33" t="n">
+        <v>1385051.612</v>
+      </c>
+      <c r="J33" t="n">
+        <v>1960137.848</v>
+      </c>
+      <c r="K33" t="n">
+        <v>598774.591</v>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Balsa Nova</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>4102307</v>
+      </c>
+      <c r="E34" t="n">
+        <v>13395</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1302016.129</v>
+      </c>
+      <c r="G34" t="n">
+        <v>97201.64999999999</v>
+      </c>
+      <c r="H34" t="n">
+        <v>103744.434</v>
+      </c>
+      <c r="I34" t="n">
+        <v>396062.227</v>
+      </c>
+      <c r="J34" t="n">
+        <v>221283.37</v>
+      </c>
+      <c r="K34" t="n">
+        <v>77568.679</v>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>Indústrias de transformação</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Califórnia</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>4103503</v>
+      </c>
+      <c r="E35" t="n">
+        <v>8710</v>
+      </c>
+      <c r="F35" t="n">
+        <v>250999.041</v>
+      </c>
+      <c r="G35" t="n">
+        <v>28817.34</v>
+      </c>
+      <c r="H35" t="n">
+        <v>67159.181</v>
+      </c>
+      <c r="I35" t="n">
+        <v>43267.043</v>
+      </c>
+      <c r="J35" t="n">
+        <v>73488.27499999999</v>
+      </c>
+      <c r="K35" t="n">
+        <v>43227.737</v>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Cambé</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>4103701</v>
+      </c>
+      <c r="E36" t="n">
+        <v>107208</v>
+      </c>
+      <c r="F36" t="n">
+        <v>6771172.732</v>
+      </c>
+      <c r="G36" t="n">
+        <v>63159.21</v>
+      </c>
+      <c r="H36" t="n">
+        <v>351440.74</v>
+      </c>
+      <c r="I36" t="n">
+        <v>1303755.414</v>
+      </c>
+      <c r="J36" t="n">
+        <v>2077406.914</v>
+      </c>
+      <c r="K36" t="n">
+        <v>498121.234</v>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Cambira</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>4103800</v>
+      </c>
+      <c r="E37" t="n">
+        <v>9460</v>
+      </c>
+      <c r="F37" t="n">
+        <v>349367.41</v>
+      </c>
+      <c r="G37" t="n">
+        <v>36931.02</v>
+      </c>
+      <c r="H37" t="n">
+        <v>76794.394</v>
+      </c>
+      <c r="I37" t="n">
+        <v>40010.564</v>
+      </c>
+      <c r="J37" t="n">
+        <v>87855.363</v>
+      </c>
+      <c r="K37" t="n">
+        <v>41751.536</v>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>Agricultura, inclusive apoio à agricultura e a pós colheita</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Ibiporã</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>4109807</v>
+      </c>
+      <c r="E38" t="n">
+        <v>51603</v>
+      </c>
+      <c r="F38" t="n">
+        <v>4037854.555</v>
+      </c>
+      <c r="G38" t="n">
+        <v>78248.45</v>
+      </c>
+      <c r="H38" t="n">
+        <v>121601.509</v>
+      </c>
+      <c r="I38" t="n">
+        <v>603664.275</v>
+      </c>
+      <c r="J38" t="n">
+        <v>1660096.847</v>
+      </c>
+      <c r="K38" t="n">
+        <v>299443.377</v>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>Comércio e reparação de veículos automotores e motocicletas</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Imbaú</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>4110078</v>
+      </c>
+      <c r="E39" t="n">
+        <v>14249</v>
+      </c>
+      <c r="F39" t="n">
+        <v>320470.89</v>
+      </c>
+      <c r="G39" t="n">
+        <v>22490.76</v>
+      </c>
+      <c r="H39" t="n">
+        <v>48196.875</v>
+      </c>
+      <c r="I39" t="n">
+        <v>34663.363</v>
+      </c>
+      <c r="J39" t="n">
+        <v>101770.875</v>
+      </c>
+      <c r="K39" t="n">
+        <v>64956.818</v>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Jandaia do Sul</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>4112108</v>
+      </c>
+      <c r="E40" t="n">
+        <v>21408</v>
+      </c>
+      <c r="F40" t="n">
+        <v>962904.172</v>
+      </c>
+      <c r="G40" t="n">
+        <v>44978.71</v>
+      </c>
+      <c r="H40" t="n">
+        <v>64850.837</v>
+      </c>
+      <c r="I40" t="n">
+        <v>142219.981</v>
+      </c>
+      <c r="J40" t="n">
+        <v>356678.031</v>
+      </c>
+      <c r="K40" t="n">
+        <v>109026.273</v>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Londrina</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>4113700</v>
+      </c>
+      <c r="E41" t="n">
+        <v>555965</v>
+      </c>
+      <c r="F41" t="n">
+        <v>27999537.379</v>
+      </c>
+      <c r="G41" t="n">
+        <v>50362.05</v>
+      </c>
+      <c r="H41" t="n">
+        <v>529678.345</v>
+      </c>
+      <c r="I41" t="n">
+        <v>4346561.46</v>
+      </c>
+      <c r="J41" t="n">
+        <v>12880750.275</v>
+      </c>
+      <c r="K41" t="n">
+        <v>2807272.707</v>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Mandaguari</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>4114203</v>
+      </c>
+      <c r="E42" t="n">
+        <v>36716</v>
+      </c>
+      <c r="F42" t="n">
+        <v>2916499.996</v>
+      </c>
+      <c r="G42" t="n">
+        <v>79434.03</v>
+      </c>
+      <c r="H42" t="n">
+        <v>248432.14</v>
+      </c>
+      <c r="I42" t="n">
+        <v>553040.216</v>
+      </c>
+      <c r="J42" t="n">
+        <v>584090.923</v>
+      </c>
+      <c r="K42" t="n">
+        <v>180325.411</v>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>Indústrias de transformação</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Marilândia do Sul</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>4114906</v>
+      </c>
+      <c r="E43" t="n">
+        <v>8677</v>
+      </c>
+      <c r="F43" t="n">
+        <v>510268.194</v>
+      </c>
+      <c r="G43" t="n">
+        <v>58806.98</v>
+      </c>
+      <c r="H43" t="n">
+        <v>248064.419</v>
+      </c>
+      <c r="I43" t="n">
+        <v>21508.931</v>
+      </c>
+      <c r="J43" t="n">
+        <v>120930.809</v>
+      </c>
+      <c r="K43" t="n">
+        <v>45343.39</v>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>Agricultura, inclusive apoio à agricultura e a pós colheita</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Mauá da Serra</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>4115754</v>
+      </c>
+      <c r="E44" t="n">
+        <v>9383</v>
+      </c>
+      <c r="F44" t="n">
+        <v>527212.083</v>
+      </c>
+      <c r="G44" t="n">
+        <v>56188.01</v>
+      </c>
+      <c r="H44" t="n">
+        <v>79540.053</v>
+      </c>
+      <c r="I44" t="n">
+        <v>84767.25199999999</v>
+      </c>
+      <c r="J44" t="n">
+        <v>110491.857</v>
+      </c>
+      <c r="K44" t="n">
+        <v>55487.846</v>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Ortigueira</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>4117305</v>
+      </c>
+      <c r="E45" t="n">
+        <v>24192</v>
+      </c>
+      <c r="F45" t="n">
+        <v>3592270.012</v>
+      </c>
+      <c r="G45" t="n">
+        <v>148490</v>
+      </c>
+      <c r="H45" t="n">
+        <v>352475.155</v>
+      </c>
+      <c r="I45" t="n">
+        <v>1584559.429</v>
+      </c>
+      <c r="J45" t="n">
+        <v>434562.281</v>
+      </c>
+      <c r="K45" t="n">
+        <v>131231.571</v>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>Indústrias de transformação</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Palmeira</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>4117701</v>
+      </c>
+      <c r="E46" t="n">
+        <v>33855</v>
+      </c>
+      <c r="F46" t="n">
+        <v>2220002.904</v>
+      </c>
+      <c r="G46" t="n">
+        <v>65573.86</v>
+      </c>
+      <c r="H46" t="n">
+        <v>447201.896</v>
+      </c>
+      <c r="I46" t="n">
+        <v>291689.448</v>
+      </c>
+      <c r="J46" t="n">
+        <v>539659.85</v>
+      </c>
+      <c r="K46" t="n">
+        <v>174051.674</v>
+      </c>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Ponta Grossa</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>4119905</v>
+      </c>
+      <c r="E47" t="n">
+        <v>358371</v>
+      </c>
+      <c r="F47" t="n">
+        <v>25583325.309</v>
+      </c>
+      <c r="G47" t="n">
+        <v>71387.82000000001</v>
+      </c>
+      <c r="H47" t="n">
+        <v>334283.776</v>
+      </c>
+      <c r="I47" t="n">
+        <v>6532267.514</v>
+      </c>
+      <c r="J47" t="n">
+        <v>7693078.622</v>
+      </c>
+      <c r="K47" t="n">
+        <v>1685113.602</v>
+      </c>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Sertaneja</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>4126405</v>
+      </c>
+      <c r="E48" t="n">
+        <v>5616</v>
+      </c>
+      <c r="F48" t="n">
+        <v>465712.008</v>
+      </c>
+      <c r="G48" t="n">
+        <v>82925.92999999999</v>
+      </c>
+      <c r="H48" t="n">
+        <v>215491.33</v>
+      </c>
+      <c r="I48" t="n">
+        <v>29692.939</v>
+      </c>
+      <c r="J48" t="n">
+        <v>108784.894</v>
+      </c>
+      <c r="K48" t="n">
+        <v>37480.26</v>
+      </c>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>Agricultura, inclusive apoio à agricultura e a pós colheita</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Sertanópolis</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>4126504</v>
+      </c>
+      <c r="E49" t="n">
+        <v>15930</v>
+      </c>
+      <c r="F49" t="n">
+        <v>863930.912</v>
+      </c>
+      <c r="G49" t="n">
+        <v>54232.95</v>
+      </c>
+      <c r="H49" t="n">
+        <v>168693.509</v>
+      </c>
+      <c r="I49" t="n">
+        <v>86586.764</v>
+      </c>
+      <c r="J49" t="n">
+        <v>274454.114</v>
+      </c>
+      <c r="K49" t="n">
+        <v>94505.08</v>
+      </c>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Tamarana</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>4126678</v>
+      </c>
+      <c r="E50" t="n">
+        <v>10707</v>
+      </c>
+      <c r="F50" t="n">
+        <v>474596.193</v>
+      </c>
+      <c r="G50" t="n">
+        <v>44325.79</v>
+      </c>
+      <c r="H50" t="n">
+        <v>147207.086</v>
+      </c>
+      <c r="I50" t="n">
+        <v>44359.441</v>
+      </c>
+      <c r="J50" t="n">
+        <v>99022.326</v>
+      </c>
+      <c r="K50" t="n">
+        <v>74328.27099999999</v>
+      </c>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>Agricultura, inclusive apoio à agricultura e a pós colheita</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Paraná Lote 3</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Tibagi</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>PR</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>4127502</v>
+      </c>
+      <c r="E51" t="n">
+        <v>19961</v>
+      </c>
+      <c r="F51" t="n">
+        <v>1448624.415</v>
+      </c>
+      <c r="G51" t="n">
+        <v>72572.74000000001</v>
+      </c>
+      <c r="H51" t="n">
+        <v>788243.754</v>
+      </c>
+      <c r="I51" t="n">
+        <v>128748.821</v>
+      </c>
+      <c r="J51" t="n">
+        <v>317181.549</v>
+      </c>
+      <c r="K51" t="n">
+        <v>121518.56</v>
+      </c>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>Agricultura, inclusive apoio à agricultura e a pós colheita</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>Amélia Rodrigues</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>2901106</v>
+      </c>
+      <c r="E52" t="n">
+        <v>24138</v>
+      </c>
+      <c r="F52" t="n">
+        <v>521349.037</v>
+      </c>
+      <c r="G52" t="n">
+        <v>21598.68</v>
+      </c>
+      <c r="H52" t="n">
+        <v>55706.71</v>
+      </c>
+      <c r="I52" t="n">
+        <v>74248.182</v>
+      </c>
+      <c r="J52" t="n">
+        <v>145817.505</v>
+      </c>
+      <c r="K52" t="n">
+        <v>105100.186</v>
+      </c>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Brejões</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>2904308</v>
+      </c>
+      <c r="E53" t="n">
+        <v>12943</v>
+      </c>
+      <c r="F53" t="n">
+        <v>168676.087</v>
+      </c>
+      <c r="G53" t="n">
+        <v>13032.22</v>
+      </c>
+      <c r="H53" t="n">
+        <v>15781.879</v>
+      </c>
+      <c r="I53" t="n">
+        <v>7227.347</v>
+      </c>
+      <c r="J53" t="n">
+        <v>47241.267</v>
+      </c>
+      <c r="K53" t="n">
+        <v>63128.731</v>
+      </c>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>Candeias</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>2906501</v>
+      </c>
+      <c r="E54" t="n">
+        <v>72382</v>
+      </c>
+      <c r="F54" t="n">
+        <v>5750025.525</v>
+      </c>
+      <c r="G54" t="n">
+        <v>79439.99000000001</v>
+      </c>
+      <c r="H54" t="n">
+        <v>16367.122</v>
+      </c>
+      <c r="I54" t="n">
+        <v>2664224.271</v>
+      </c>
+      <c r="J54" t="n">
+        <v>2411306.041</v>
+      </c>
+      <c r="K54" t="n">
+        <v>452597.51</v>
+      </c>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>Indústrias de transformação</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Cândido Sales</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>2906709</v>
+      </c>
+      <c r="E55" t="n">
+        <v>25247</v>
+      </c>
+      <c r="F55" t="n">
+        <v>289056.859</v>
+      </c>
+      <c r="G55" t="n">
+        <v>11449.16</v>
+      </c>
+      <c r="H55" t="n">
+        <v>12897.561</v>
+      </c>
+      <c r="I55" t="n">
+        <v>12968.724</v>
+      </c>
+      <c r="J55" t="n">
+        <v>90924.53999999999</v>
+      </c>
+      <c r="K55" t="n">
+        <v>109249.365</v>
+      </c>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>Feira de Santana</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>2910800</v>
+      </c>
+      <c r="E56" t="n">
+        <v>616272</v>
+      </c>
+      <c r="F56" t="n">
+        <v>21846454.667</v>
+      </c>
+      <c r="G56" t="n">
+        <v>35449.37</v>
+      </c>
+      <c r="H56" t="n">
+        <v>85543.288</v>
+      </c>
+      <c r="I56" t="n">
+        <v>3699324.796</v>
+      </c>
+      <c r="J56" t="n">
+        <v>8594182.423</v>
+      </c>
+      <c r="K56" t="n">
+        <v>1931140.63</v>
+      </c>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Jaguaquara</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>2917607</v>
+      </c>
+      <c r="E57" t="n">
+        <v>45964</v>
+      </c>
+      <c r="F57" t="n">
+        <v>807068.769</v>
+      </c>
+      <c r="G57" t="n">
+        <v>17558.71</v>
+      </c>
+      <c r="H57" t="n">
+        <v>69162.224</v>
+      </c>
+      <c r="I57" t="n">
+        <v>33759.243</v>
+      </c>
+      <c r="J57" t="n">
+        <v>297888.225</v>
+      </c>
+      <c r="K57" t="n">
+        <v>207180.099</v>
+      </c>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>Jequié</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>2918001</v>
+      </c>
+      <c r="E58" t="n">
+        <v>158813</v>
+      </c>
+      <c r="F58" t="n">
+        <v>3882706.96</v>
+      </c>
+      <c r="G58" t="n">
+        <v>24448.29</v>
+      </c>
+      <c r="H58" t="n">
+        <v>77837.90700000001</v>
+      </c>
+      <c r="I58" t="n">
+        <v>389021.957</v>
+      </c>
+      <c r="J58" t="n">
+        <v>1648896.469</v>
+      </c>
+      <c r="K58" t="n">
+        <v>627446.705</v>
+      </c>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Manoel Vitorino</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>2920403</v>
+      </c>
+      <c r="E59" t="n">
+        <v>13860</v>
+      </c>
+      <c r="F59" t="n">
+        <v>165431.588</v>
+      </c>
+      <c r="G59" t="n">
+        <v>11935.9</v>
+      </c>
+      <c r="H59" t="n">
+        <v>35511.583</v>
+      </c>
+      <c r="I59" t="n">
+        <v>5847.384</v>
+      </c>
+      <c r="J59" t="n">
+        <v>34710.363</v>
+      </c>
+      <c r="K59" t="n">
+        <v>57281.231</v>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>Milagres</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>2921302</v>
+      </c>
+      <c r="E60" t="n">
+        <v>11071</v>
+      </c>
+      <c r="F60" t="n">
+        <v>181064.199</v>
+      </c>
+      <c r="G60" t="n">
+        <v>16354.82</v>
+      </c>
+      <c r="H60" t="n">
+        <v>2664.851</v>
+      </c>
+      <c r="I60" t="n">
+        <v>6721.668</v>
+      </c>
+      <c r="J60" t="n">
+        <v>68972.57799999999</v>
+      </c>
+      <c r="K60" t="n">
+        <v>47706.528</v>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Planalto</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>2925006</v>
+      </c>
+      <c r="E61" t="n">
+        <v>23334</v>
+      </c>
+      <c r="F61" t="n">
+        <v>324874.126</v>
+      </c>
+      <c r="G61" t="n">
+        <v>13922.78</v>
+      </c>
+      <c r="H61" t="n">
+        <v>45780.423</v>
+      </c>
+      <c r="I61" t="n">
+        <v>21524.458</v>
+      </c>
+      <c r="J61" t="n">
+        <v>113614.334</v>
+      </c>
+      <c r="K61" t="n">
+        <v>102036.748</v>
+      </c>
+      <c r="L61" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Poções</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>2925105</v>
+      </c>
+      <c r="E62" t="n">
+        <v>48293</v>
+      </c>
+      <c r="F62" t="n">
+        <v>681871.458</v>
+      </c>
+      <c r="G62" t="n">
+        <v>14119.47</v>
+      </c>
+      <c r="H62" t="n">
+        <v>32742.63</v>
+      </c>
+      <c r="I62" t="n">
+        <v>33353.78</v>
+      </c>
+      <c r="J62" t="n">
+        <v>274593.046</v>
+      </c>
+      <c r="K62" t="n">
+        <v>172522.219</v>
+      </c>
+      <c r="L62" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Rafael Jambeiro</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>2925956</v>
+      </c>
+      <c r="E63" t="n">
+        <v>19662</v>
+      </c>
+      <c r="F63" t="n">
+        <v>422266.249</v>
+      </c>
+      <c r="G63" t="n">
+        <v>21476.26</v>
+      </c>
+      <c r="H63" t="n">
+        <v>17641.085</v>
+      </c>
+      <c r="I63" t="n">
+        <v>14111.758</v>
+      </c>
+      <c r="J63" t="n">
+        <v>209824.895</v>
+      </c>
+      <c r="K63" t="n">
+        <v>91433.83199999999</v>
+      </c>
+      <c r="L63" t="inlineStr">
+        <is>
+          <t>Comércio e reparação de veículos automotores e motocicletas</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Salvador</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>2927408</v>
+      </c>
+      <c r="E64" t="n">
+        <v>2417678</v>
+      </c>
+      <c r="F64" t="n">
+        <v>76698777.21799999</v>
+      </c>
+      <c r="G64" t="n">
+        <v>31724.15</v>
+      </c>
+      <c r="H64" t="n">
+        <v>52696.652</v>
+      </c>
+      <c r="I64" t="n">
+        <v>7154630.575</v>
+      </c>
+      <c r="J64" t="n">
+        <v>38143695.917</v>
+      </c>
+      <c r="K64" t="n">
+        <v>8893534.727</v>
+      </c>
+      <c r="L64" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Santo Estêvão</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2928802</v>
+      </c>
+      <c r="E65" t="n">
+        <v>52276</v>
+      </c>
+      <c r="F65" t="n">
+        <v>1295366.193</v>
+      </c>
+      <c r="G65" t="n">
+        <v>24779.37</v>
+      </c>
+      <c r="H65" t="n">
+        <v>17037.175</v>
+      </c>
+      <c r="I65" t="n">
+        <v>173012.285</v>
+      </c>
+      <c r="J65" t="n">
+        <v>384809.454</v>
+      </c>
+      <c r="K65" t="n">
+        <v>212675.46</v>
+      </c>
+      <c r="L65" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>São Sebastião do Passé</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>2929503</v>
+      </c>
+      <c r="E66" t="n">
+        <v>40958</v>
+      </c>
+      <c r="F66" t="n">
+        <v>957089.48</v>
+      </c>
+      <c r="G66" t="n">
+        <v>23367.58</v>
+      </c>
+      <c r="H66" t="n">
+        <v>25522.585</v>
+      </c>
+      <c r="I66" t="n">
+        <v>261854.884</v>
+      </c>
+      <c r="J66" t="n">
+        <v>262010.108</v>
+      </c>
+      <c r="K66" t="n">
+        <v>183968.809</v>
+      </c>
+      <c r="L66" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Simões Filho</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>2930709</v>
+      </c>
+      <c r="E67" t="n">
+        <v>114559</v>
+      </c>
+      <c r="F67" t="n">
+        <v>8508321.271</v>
+      </c>
+      <c r="G67" t="n">
+        <v>74270.21000000001</v>
+      </c>
+      <c r="H67" t="n">
+        <v>11984.8</v>
+      </c>
+      <c r="I67" t="n">
+        <v>2200927.709</v>
+      </c>
+      <c r="J67" t="n">
+        <v>2175567.098</v>
+      </c>
+      <c r="K67" t="n">
+        <v>593739.353</v>
+      </c>
+      <c r="L67" t="inlineStr">
+        <is>
+          <t>Indústrias de transformação</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Rota 2 de Julho</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Vitória da Conquista</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>BA</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>2933307</v>
+      </c>
+      <c r="E68" t="n">
+        <v>370879</v>
+      </c>
+      <c r="F68" t="n">
+        <v>12666570.589</v>
+      </c>
+      <c r="G68" t="n">
+        <v>34152.84</v>
+      </c>
+      <c r="H68" t="n">
+        <v>188037.51</v>
+      </c>
+      <c r="I68" t="n">
+        <v>1219365.299</v>
+      </c>
+      <c r="J68" t="n">
+        <v>4319364.453</v>
+      </c>
+      <c r="K68" t="n">
+        <v>1321865.48</v>
+      </c>
+      <c r="L68" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Ariquemes</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>1100023</v>
+      </c>
+      <c r="E69" t="n">
+        <v>96833</v>
+      </c>
+      <c r="F69" t="n">
+        <v>4383815.338</v>
+      </c>
+      <c r="G69" t="n">
+        <v>45271.91</v>
+      </c>
+      <c r="H69" t="n">
+        <v>293000.779</v>
+      </c>
+      <c r="I69" t="n">
+        <v>407674.509</v>
+      </c>
+      <c r="J69" t="n">
+        <v>1307976.899</v>
+      </c>
+      <c r="K69" t="n">
+        <v>782306.216</v>
+      </c>
+      <c r="L69" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cacoal</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1100049</v>
+      </c>
+      <c r="E70" t="n">
+        <v>86887</v>
+      </c>
+      <c r="F70" t="n">
+        <v>3848467.896</v>
+      </c>
+      <c r="G70" t="n">
+        <v>44292.79</v>
+      </c>
+      <c r="H70" t="n">
+        <v>341314.544</v>
+      </c>
+      <c r="I70" t="n">
+        <v>236801.003</v>
+      </c>
+      <c r="J70" t="n">
+        <v>1200653.615</v>
+      </c>
+      <c r="K70" t="n">
+        <v>629109.371</v>
+      </c>
+      <c r="L70" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Jaru</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>1100114</v>
+      </c>
+      <c r="E71" t="n">
+        <v>50591</v>
+      </c>
+      <c r="F71" t="n">
+        <v>2515557.725</v>
+      </c>
+      <c r="G71" t="n">
+        <v>49723.42</v>
+      </c>
+      <c r="H71" t="n">
+        <v>280710.555</v>
+      </c>
+      <c r="I71" t="n">
+        <v>177622.679</v>
+      </c>
+      <c r="J71" t="n">
+        <v>688454.672</v>
+      </c>
+      <c r="K71" t="n">
+        <v>379859.774</v>
+      </c>
+      <c r="L71" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Ji-Paraná</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>1100122</v>
+      </c>
+      <c r="E72" t="n">
+        <v>124333</v>
+      </c>
+      <c r="F72" t="n">
+        <v>5824472.224</v>
+      </c>
+      <c r="G72" t="n">
+        <v>46845.75</v>
+      </c>
+      <c r="H72" t="n">
+        <v>206344.829</v>
+      </c>
+      <c r="I72" t="n">
+        <v>502237.665</v>
+      </c>
+      <c r="J72" t="n">
+        <v>1926052.214</v>
+      </c>
+      <c r="K72" t="n">
+        <v>876138.6360000001</v>
+      </c>
+      <c r="L72" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Ouro Preto do Oeste</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1100155</v>
+      </c>
+      <c r="E73" t="n">
+        <v>35044</v>
+      </c>
+      <c r="F73" t="n">
+        <v>1275478.843</v>
+      </c>
+      <c r="G73" t="n">
+        <v>36396.5</v>
+      </c>
+      <c r="H73" t="n">
+        <v>216209.007</v>
+      </c>
+      <c r="I73" t="n">
+        <v>71310.999</v>
+      </c>
+      <c r="J73" t="n">
+        <v>352571.686</v>
+      </c>
+      <c r="K73" t="n">
+        <v>249016.476</v>
+      </c>
+      <c r="L73" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Pimenta Bueno</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>1100189</v>
+      </c>
+      <c r="E74" t="n">
+        <v>35079</v>
+      </c>
+      <c r="F74" t="n">
+        <v>2124340.165</v>
+      </c>
+      <c r="G74" t="n">
+        <v>60558.74</v>
+      </c>
+      <c r="H74" t="n">
+        <v>297492.054</v>
+      </c>
+      <c r="I74" t="n">
+        <v>207693.244</v>
+      </c>
+      <c r="J74" t="n">
+        <v>550815.52</v>
+      </c>
+      <c r="K74" t="n">
+        <v>280779.155</v>
+      </c>
+      <c r="L74" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Porto Velho</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>1100205</v>
+      </c>
+      <c r="E75" t="n">
+        <v>460434</v>
+      </c>
+      <c r="F75" t="n">
+        <v>25402193.434</v>
+      </c>
+      <c r="G75" t="n">
+        <v>55170.11</v>
+      </c>
+      <c r="H75" t="n">
+        <v>1041284.612</v>
+      </c>
+      <c r="I75" t="n">
+        <v>4625035.281</v>
+      </c>
+      <c r="J75" t="n">
+        <v>7555290.353</v>
+      </c>
+      <c r="K75" t="n">
+        <v>3983359.174</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Demais serviços</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Presidente Médici</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>1100254</v>
+      </c>
+      <c r="E76" t="n">
+        <v>19327</v>
+      </c>
+      <c r="F76" t="n">
+        <v>776280.726</v>
+      </c>
+      <c r="G76" t="n">
+        <v>40165.61</v>
+      </c>
+      <c r="H76" t="n">
+        <v>183438.443</v>
+      </c>
+      <c r="I76" t="n">
+        <v>50709.564</v>
+      </c>
+      <c r="J76" t="n">
+        <v>140127.735</v>
+      </c>
+      <c r="K76" t="n">
+        <v>134436.852</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Pecuária, inclusive apoio à pecuária</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Vilhena</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>1100304</v>
+      </c>
+      <c r="E77" t="n">
+        <v>95832</v>
+      </c>
+      <c r="F77" t="n">
+        <v>5115785.079</v>
+      </c>
+      <c r="G77" t="n">
+        <v>53382.85</v>
+      </c>
+      <c r="H77" t="n">
+        <v>674880.42</v>
+      </c>
+      <c r="I77" t="n">
+        <v>369205.556</v>
+      </c>
+      <c r="J77" t="n">
+        <v>1712252.035</v>
+      </c>
+      <c r="K77" t="n">
+        <v>777251.976</v>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Comércio e reparação de veículos automotores e motocicletas</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Candeias do Jamari</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>1100809</v>
+      </c>
+      <c r="E78" t="n">
+        <v>22310</v>
+      </c>
+      <c r="F78" t="n">
+        <v>1001610.328</v>
+      </c>
+      <c r="G78" t="n">
+        <v>44895.13</v>
+      </c>
+      <c r="H78" t="n">
+        <v>141452.035</v>
+      </c>
+      <c r="I78" t="n">
+        <v>133642.718</v>
+      </c>
+      <c r="J78" t="n">
+        <v>138507.479</v>
+      </c>
+      <c r="K78" t="n">
+        <v>204881.885</v>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Rota Agro Norte (CN5)</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Itapuã do Oeste</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>RO</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>1101104</v>
+      </c>
+      <c r="E79" t="n">
+        <v>8548</v>
+      </c>
+      <c r="F79" t="n">
+        <v>340162.494</v>
+      </c>
+      <c r="G79" t="n">
+        <v>39794.4</v>
+      </c>
+      <c r="H79" t="n">
+        <v>65084.768</v>
+      </c>
+      <c r="I79" t="n">
+        <v>14562.761</v>
+      </c>
+      <c r="J79" t="n">
+        <v>39827.234</v>
+      </c>
+      <c r="K79" t="n">
+        <v>79560.32399999999</v>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Administração, defesa, educação e saúde públicas e seguridade social</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>